<commit_message>
fix(import): NocoBase branding - Sheet1, no ID column, RU-title xlsx for column mapping
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/import/nocobase-subscription_branding.xlsx
+++ b/import/nocobase-subscription_branding.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="subscription_branding" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,55 +413,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>subscriptionTitle</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>subscriptionTitle</t>
+          <t>supportUrl</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>supportUrl</t>
+          <t>profileUrl</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>profileUrl</t>
+          <t>announcement</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
-        <is>
-          <t>announcement</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
     </row>
     <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>VL</t>
+        </is>
+      </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>VL</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
           <t>https://t.me/VL_VPNbot</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="b">
+      <c r="E2" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: subscription_branding active as text for NocoBase import; parse string active in bot
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/import/nocobase-subscription_branding.xlsx
+++ b/import/nocobase-subscription_branding.xlsx
@@ -413,56 +413,51 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>subscriptionTitle</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>subscriptionTitle</t>
+          <t>supportUrl</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>supportUrl</t>
+          <t>profileUrl</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>profileUrl</t>
+          <t>announcement</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
-        <is>
-          <t>announcement</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
     </row>
     <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>VL</t>
+        </is>
+      </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>VL</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
           <t>https://t.me/VL_VPNbot</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="b">
-        <v>1</v>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: prepend ID column for NocoBase subscription_branding import
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/import/nocobase-subscription_branding.xlsx
+++ b/import/nocobase-subscription_branding.xlsx
@@ -413,48 +413,53 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>subscriptionTitle</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>supportUrl</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>profileUrl</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>announcement</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>VL</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>https://t.me/VL_VPNbot</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>true</t>
         </is>

</xml_diff>